<commit_message>
fix(main): reset freeze panes to A3 — was stuck at A217 blocking scroll
The copy_main_sheet() function was copying the source file's saved view
position (A217) instead of forcing the correct freeze at row 3.
Fixed the live file and patched cmf_import_pm_updates.py to always
set freeze_panes='A3' regardless of what the source file had.

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CMF WIP - Schedule.xlsx
+++ b/CMF WIP - Schedule.xlsx
@@ -6647,6 +6647,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6677,6 +6680,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6707,6 +6713,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6737,6 +6746,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6767,6 +6779,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6797,6 +6812,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6827,6 +6845,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6857,6 +6878,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6887,6 +6911,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6917,6 +6944,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6947,6 +6977,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6977,6 +7010,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7007,6 +7043,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7037,6 +7076,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7067,6 +7109,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7097,6 +7142,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7127,6 +7175,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7157,6 +7208,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7187,6 +7241,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7217,6 +7274,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7247,6 +7307,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7277,6 +7340,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7307,6 +7373,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7337,6 +7406,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7367,6 +7439,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7397,6 +7472,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7427,6 +7505,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7457,6 +7538,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7487,6 +7571,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7517,6 +7604,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7547,6 +7637,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7577,6 +7670,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7607,6 +7703,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7637,6 +7736,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7667,6 +7769,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7697,6 +7802,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7727,6 +7835,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7757,6 +7868,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7787,6 +7901,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7817,6 +7934,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7847,6 +7967,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7877,6 +8000,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7907,6 +8033,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7937,6 +8066,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7967,6 +8099,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -7997,6 +8132,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8027,6 +8165,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8057,6 +8198,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8087,6 +8231,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8117,6 +8264,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8147,6 +8297,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8177,6 +8330,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8207,6 +8363,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8237,6 +8396,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8267,6 +8429,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8297,6 +8462,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8327,6 +8495,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8357,6 +8528,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8387,6 +8561,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8417,6 +8594,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8447,6 +8627,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8477,6 +8660,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8507,6 +8693,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8537,6 +8726,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8567,6 +8759,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8597,6 +8792,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8627,6 +8825,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8657,6 +8858,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8687,6 +8891,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8717,6 +8924,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8747,6 +8957,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8777,6 +8990,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8807,6 +9023,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8837,6 +9056,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8867,6 +9089,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8897,6 +9122,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8927,6 +9155,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8957,6 +9188,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -8987,6 +9221,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9017,6 +9254,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9047,6 +9287,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9077,6 +9320,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9107,6 +9353,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9137,6 +9386,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9167,6 +9419,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9197,6 +9452,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9227,6 +9485,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9257,6 +9518,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9287,6 +9551,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9317,6 +9584,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9347,6 +9617,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9377,6 +9650,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9407,6 +9683,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9437,6 +9716,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9467,6 +9749,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9497,6 +9782,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9527,6 +9815,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9557,6 +9848,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9587,6 +9881,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9617,6 +9914,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9647,6 +9947,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9677,6 +9980,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9707,6 +10013,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9737,6 +10046,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9767,6 +10079,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9797,6 +10112,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9827,6 +10145,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9857,6 +10178,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9887,6 +10211,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9917,6 +10244,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9947,6 +10277,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -9977,6 +10310,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10007,6 +10343,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10037,6 +10376,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10067,6 +10409,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10097,6 +10442,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10127,6 +10475,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10157,6 +10508,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10187,6 +10541,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10217,6 +10574,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10247,6 +10607,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10277,6 +10640,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10307,6 +10673,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10337,6 +10706,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10367,6 +10739,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10397,6 +10772,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10427,6 +10805,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10457,6 +10838,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10487,6 +10871,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10517,6 +10904,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10547,6 +10937,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10582,6 +10975,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10612,6 +11008,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10642,6 +11041,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10672,6 +11074,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10702,6 +11107,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10732,6 +11140,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10762,6 +11173,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10792,6 +11206,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10822,6 +11239,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10852,6 +11272,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10882,6 +11305,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10912,6 +11338,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10942,6 +11371,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -10972,6 +11404,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11002,6 +11437,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11032,6 +11470,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11062,6 +11503,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11092,6 +11536,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11122,6 +11569,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11152,6 +11602,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11182,6 +11635,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11212,6 +11668,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11242,6 +11701,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11272,6 +11734,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11302,6 +11767,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11332,6 +11800,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11362,6 +11833,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11392,6 +11866,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11422,6 +11899,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11452,6 +11932,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11482,6 +11965,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11512,6 +11998,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11542,6 +12031,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11572,6 +12064,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11602,6 +12097,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11632,6 +12130,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11662,6 +12163,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11692,6 +12196,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11722,6 +12229,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11752,6 +12262,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11782,6 +12295,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11812,6 +12328,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11842,6 +12361,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11872,6 +12394,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11902,6 +12427,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11932,6 +12460,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11962,6 +12493,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -11992,6 +12526,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12022,6 +12559,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12052,6 +12592,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12082,6 +12625,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12112,6 +12658,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12142,6 +12691,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12172,6 +12724,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12202,6 +12757,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12232,6 +12790,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12262,6 +12823,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12292,6 +12856,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12322,6 +12889,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12352,6 +12922,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12382,6 +12955,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12412,6 +12988,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12442,6 +13021,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12472,6 +13054,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12502,6 +13087,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12532,6 +13120,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12562,6 +13153,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12592,6 +13186,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12622,6 +13219,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12652,6 +13252,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12682,6 +13285,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12712,6 +13318,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12742,6 +13351,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12772,6 +13384,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12802,6 +13417,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12832,6 +13450,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12862,6 +13483,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12892,6 +13516,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12922,6 +13549,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12952,6 +13582,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -12982,6 +13615,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13012,6 +13648,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13042,6 +13681,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13072,6 +13714,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13102,6 +13747,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13132,6 +13780,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13162,6 +13813,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13192,6 +13846,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13222,6 +13879,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13252,6 +13912,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13282,6 +13945,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13312,6 +13978,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13342,6 +14011,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13372,6 +14044,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13402,6 +14077,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13432,6 +14110,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13462,6 +14143,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13492,6 +14176,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13522,6 +14209,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13552,6 +14242,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13582,6 +14275,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13612,6 +14308,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13642,6 +14341,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13672,6 +14374,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13702,6 +14407,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13732,6 +14440,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13762,6 +14473,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13792,6 +14506,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13822,6 +14539,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13852,6 +14572,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13882,6 +14605,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13912,6 +14638,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13942,6 +14671,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -13972,6 +14704,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14002,6 +14737,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14032,6 +14770,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14062,6 +14803,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14092,6 +14836,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14122,6 +14869,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14152,6 +14902,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14182,6 +14935,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14212,6 +14968,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14242,6 +15001,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14272,6 +15034,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14302,6 +15067,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14332,6 +15100,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14362,6 +15133,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14392,6 +15166,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14422,6 +15199,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14452,6 +15232,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14482,6 +15265,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14512,6 +15298,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14542,6 +15331,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14572,6 +15364,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14602,6 +15397,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14632,6 +15430,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14662,6 +15463,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14692,6 +15496,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14722,6 +15529,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14752,6 +15562,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14782,6 +15595,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14812,6 +15628,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14842,6 +15661,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14872,6 +15694,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14902,6 +15727,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14932,6 +15760,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14962,6 +15793,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -14992,6 +15826,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15022,6 +15859,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15052,6 +15892,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15082,6 +15925,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15112,6 +15958,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15142,6 +15991,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15172,6 +16024,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15202,6 +16057,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15232,6 +16090,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15262,6 +16123,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15292,6 +16156,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15322,6 +16189,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15352,6 +16222,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15382,6 +16255,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15412,6 +16288,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15442,6 +16321,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15472,6 +16354,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15502,6 +16387,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15532,6 +16420,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15562,6 +16453,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15592,6 +16486,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15622,6 +16519,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15652,6 +16552,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15682,6 +16585,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15712,6 +16618,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15742,6 +16651,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15772,6 +16684,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15802,6 +16717,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15832,6 +16750,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15862,6 +16783,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15892,6 +16816,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15922,6 +16849,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15952,6 +16882,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -15982,6 +16915,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16012,6 +16948,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16042,6 +16981,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16072,6 +17014,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16102,6 +17047,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16132,6 +17080,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16162,6 +17113,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16192,6 +17146,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16222,6 +17179,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16252,6 +17212,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16282,6 +17245,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16312,6 +17278,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16342,6 +17311,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16372,6 +17344,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16402,6 +17377,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16432,6 +17410,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16462,6 +17443,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16492,6 +17476,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16522,6 +17509,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16552,6 +17542,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16582,6 +17575,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16612,6 +17608,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16647,6 +17646,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16677,6 +17679,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16707,6 +17712,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16737,6 +17745,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16767,6 +17778,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16797,6 +17811,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16827,6 +17844,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16857,6 +17877,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16887,6 +17910,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16917,6 +17943,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16947,6 +17976,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -16977,6 +18009,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17007,6 +18042,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17037,6 +18075,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17067,6 +18108,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17097,6 +18141,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17127,6 +18174,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17157,6 +18207,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17187,6 +18240,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17217,6 +18273,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17247,6 +18306,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17277,6 +18339,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17307,6 +18372,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17337,6 +18405,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17367,6 +18438,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17397,6 +18471,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17427,6 +18504,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17457,6 +18537,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17487,6 +18570,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17517,6 +18603,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -17547,6 +18636,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>